<commit_message>
feat(mop): add static context and rex brief zone before phase 1 in fiche mop
</commit_message>
<xml_diff>
--- a/incidents-otn-oob-v2.xlsx
+++ b/incidents-otn-oob-v2.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="19">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,66 +64,66 @@
       <sz val="8"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00B0BEC5"/>
       <sz val="9"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="13"/>
-    </font>
-    <font>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="9"/>
-    </font>
-    <font>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00607D8B"/>
       <sz val="8"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001F5C8B"/>
       <sz val="9"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00000000"/>
       <sz val="9"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00B71C1C"/>
       <sz val="9"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="9"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="28">
+  <fills count="31">
     <fill>
       <patternFill/>
     </fill>
@@ -242,6 +242,21 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="004E342E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006D4C41"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="003A5A8A"/>
       </patternFill>
     </fill>
@@ -301,7 +316,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -410,43 +425,57 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="21" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="27" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="25" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="28" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="25" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="28" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="27" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="30" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="27" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6914,7 +6943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E152"/>
+  <dimension ref="A1:E160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6934,7 +6963,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="36" t="inlineStr">
         <is>
-          <t>Zones jaunes = saisie obligatoire · Zones vertes = résultats · Zones grises = lecture seule</t>
+          <t>Zones jaunes = saisie obligatoire · Zones vertes = résultats · Zones ambre = description/REX · Gris = lecture seule</t>
         </is>
       </c>
     </row>
@@ -6968,7 +6997,7 @@
       <c r="B6" s="41" t="n"/>
       <c r="C6" s="40" t="inlineStr">
         <is>
-          <t>ID MOP (auto ou manuel)</t>
+          <t>ID MOP</t>
         </is>
       </c>
       <c r="D6" s="41" t="n"/>
@@ -7000,7 +7029,7 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="40" t="inlineStr">
         <is>
-          <t>Criticité (MINEUR/MAJEUR/CRITIQUE)</t>
+          <t>Criticité</t>
         </is>
       </c>
       <c r="B8" s="41" t="n"/>
@@ -7076,19 +7105,11 @@
       <c r="D12" s="41" t="n"/>
       <c r="E12" s="37" t="n"/>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="40" t="inlineStr">
-        <is>
-          <t>Alarme Lightsoft observée</t>
-        </is>
-      </c>
-      <c r="B13" s="41" t="n"/>
-      <c r="C13" s="40" t="inlineStr">
-        <is>
-          <t>Alarme Vizee observée</t>
-        </is>
-      </c>
-      <c r="D13" s="41" t="n"/>
+    <row r="13" ht="6" customHeight="1">
+      <c r="A13" s="37" t="n"/>
+      <c r="B13" s="37" t="n"/>
+      <c r="C13" s="37" t="n"/>
+      <c r="D13" s="37" t="n"/>
       <c r="E13" s="37" t="n"/>
     </row>
     <row r="14" ht="6" customHeight="1">
@@ -7099,644 +7120,580 @@
       <c r="E14" s="37" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="38" t="inlineStr">
+      <c r="A15" s="43" t="inlineStr">
+        <is>
+          <t>CONTEXTE — Description, Symptômes connus &amp; Cause probable</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="14" customHeight="1">
+      <c r="A16" s="44" t="inlineStr">
+        <is>
+          <t>À rédiger une fois lors de la création du MOP — basé sur l'historique terrain. Guider le technicien avant l'intervention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="52" customHeight="1">
+      <c r="A17" s="45" t="inlineStr">
+        <is>
+          <t>Description de l'incident</t>
+        </is>
+      </c>
+      <c r="B17" s="46" t="n"/>
+      <c r="E17" s="47" t="inlineStr">
+        <is>
+          <t>Expliquer en 2-3 phrases ce que représente cet incident, son contexte opérationnel et son impact typique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="52" customHeight="1">
+      <c r="A18" s="45" t="inlineStr">
+        <is>
+          <t>Symptômes observés
+(typiquement)</t>
+        </is>
+      </c>
+      <c r="B18" s="46" t="n"/>
+      <c r="E18" s="47" t="inlineStr">
+        <is>
+          <t>Ce que le technicien va voir sur Lightsoft / Vizee. Alarmes, couleurs NE, messages d'erreur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="44" customHeight="1">
+      <c r="A19" s="45" t="inlineStr">
+        <is>
+          <t>Cause probable principale</t>
+        </is>
+      </c>
+      <c r="B19" s="46" t="n"/>
+      <c r="E19" s="47" t="inlineStr">
+        <is>
+          <t>Cause la plus fréquente identifiée sur le terrain. Base sur les REX précédents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="44" customHeight="1">
+      <c r="A20" s="45" t="inlineStr">
+        <is>
+          <t>Causes secondaires
+possibles</t>
+        </is>
+      </c>
+      <c r="B20" s="46" t="n"/>
+      <c r="E20" s="47" t="inlineStr">
+        <is>
+          <t>Autres causes observées moins fréquemment. À explorer si la cause principale est écartée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="52" customHeight="1">
+      <c r="A21" s="45" t="inlineStr">
+        <is>
+          <t>Points d'attention
+&amp; règles critiques</t>
+        </is>
+      </c>
+      <c r="B21" s="46" t="n"/>
+      <c r="E21" s="47" t="inlineStr">
+        <is>
+          <t>⚠ Ce qu'il ne faut pas faire. Erreurs passées. Règles LOI OP applicables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="45" t="inlineStr">
+        <is>
+          <t>Notes terrain
+(REX cumulé)</t>
+        </is>
+      </c>
+      <c r="B22" s="46" t="n"/>
+      <c r="E22" s="47" t="inlineStr">
+        <is>
+          <t>Zone libre — à compléter après chaque incident. Observations, astuces, cas particuliers rencontrés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="6" customHeight="1">
+      <c r="A23" s="37" t="n"/>
+      <c r="B23" s="37" t="n"/>
+      <c r="C23" s="37" t="n"/>
+      <c r="D23" s="37" t="n"/>
+      <c r="E23" s="37" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="38" t="inlineStr">
         <is>
           <t>PHASE 1 — QUALIFICATION</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="14" customHeight="1">
-      <c r="A16" s="39" t="inlineStr">
+    <row r="25" ht="14" customHeight="1">
+      <c r="A25" s="39" t="inlineStr">
         <is>
           <t>SOP-01 · Toujours exécutée</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="43" t="inlineStr">
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="48" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  SOP-01 — Qualification initiale alarme</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="44" t="inlineStr">
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 1</t>
         </is>
       </c>
-      <c r="B18" s="45" t="inlineStr">
+      <c r="B27" s="50" t="inlineStr">
         <is>
           <t>Ouvrir Lightsoft ET Vizee simultanément</t>
         </is>
       </c>
-      <c r="C18" s="40" t="inlineStr">
+      <c r="C27" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D18" s="46" t="n"/>
-      <c r="E18" s="42" t="inlineStr">
+      <c r="D27" s="51" t="n"/>
+      <c r="E27" s="42" t="inlineStr">
         <is>
           <t>Outil : Lightsoft / Vizee</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="44" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 2</t>
         </is>
       </c>
-      <c r="B19" s="45" t="inlineStr">
+      <c r="B28" s="50" t="inlineStr">
         <is>
           <t>Identifier la couleur des NE : Bleu/gris → supervision seule · Rouge/alarme → trafic impacté</t>
         </is>
       </c>
-      <c r="C19" s="40" t="inlineStr">
+      <c r="C28" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D19" s="46" t="n"/>
-      <c r="E19" s="42" t="inlineStr">
+      <c r="D28" s="51" t="n"/>
+      <c r="E28" s="42" t="inlineStr">
         <is>
           <t>Outil : Lightsoft</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="44" t="inlineStr">
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 3</t>
         </is>
       </c>
-      <c r="B20" s="45" t="inlineStr">
+      <c r="B29" s="50" t="inlineStr">
         <is>
           <t>Compter les alarmes simultanées : 1 isolée vs avalanche = diagnostic différent</t>
         </is>
       </c>
-      <c r="C20" s="40" t="inlineStr">
+      <c r="C29" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D20" s="46" t="n"/>
-      <c r="E20" s="42" t="inlineStr">
+      <c r="D29" s="51" t="n"/>
+      <c r="E29" s="42" t="inlineStr">
         <is>
           <t>Outil : Vizee</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="44" t="inlineStr">
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 4</t>
         </is>
       </c>
-      <c r="B21" s="45" t="inlineStr">
+      <c r="B30" s="50" t="inlineStr">
         <is>
           <t>Croiser avec journal des opérations : travaux en cours ? maintenance annoncée ?</t>
         </is>
       </c>
-      <c r="C21" s="40" t="inlineStr">
+      <c r="C30" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D21" s="46" t="n"/>
-      <c r="E21" s="42" t="inlineStr">
+      <c r="D30" s="51" t="n"/>
+      <c r="E30" s="42" t="inlineStr">
         <is>
           <t>Outil : Journal interne</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="44" t="inlineStr">
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 5</t>
         </is>
       </c>
-      <c r="B22" s="45" t="inlineStr">
+      <c r="B31" s="50" t="inlineStr">
         <is>
           <t>Horodater l'alarme (heure de début)</t>
         </is>
       </c>
-      <c r="C22" s="40" t="inlineStr">
+      <c r="C31" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D22" s="46" t="n"/>
-      <c r="E22" s="42" t="inlineStr">
+      <c r="D31" s="51" t="n"/>
+      <c r="E31" s="42" t="inlineStr">
         <is>
           <t>Outil : Vizee / Lightsoft</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="47" t="inlineStr">
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="52" t="inlineStr">
         <is>
           <t>⚠  NE bleu/gris ≠ perte de trafic — ne pas escalader avant confirmation</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="40" t="inlineStr">
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="40" t="inlineStr">
         <is>
           <t>Impact évalué</t>
         </is>
       </c>
-      <c r="B24" s="41" t="n"/>
-      <c r="C24" s="40" t="inlineStr">
+      <c r="B33" s="41" t="n"/>
+      <c r="C33" s="40" t="inlineStr">
         <is>
           <t>Criticité confirmée</t>
         </is>
       </c>
-      <c r="D24" s="41" t="n"/>
-      <c r="E24" s="37" t="n"/>
-    </row>
-    <row r="25" ht="6" customHeight="1">
-      <c r="A25" s="37" t="n"/>
-      <c r="B25" s="37" t="n"/>
-      <c r="C25" s="37" t="n"/>
-      <c r="D25" s="37" t="n"/>
-      <c r="E25" s="37" t="n"/>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="38" t="inlineStr">
+      <c r="D33" s="41" t="n"/>
+      <c r="E33" s="37" t="n"/>
+    </row>
+    <row r="34" ht="6" customHeight="1">
+      <c r="A34" s="37" t="n"/>
+      <c r="B34" s="37" t="n"/>
+      <c r="C34" s="37" t="n"/>
+      <c r="D34" s="37" t="n"/>
+      <c r="E34" s="37" t="n"/>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="38" t="inlineStr">
         <is>
           <t>PHASE 2 — DIAGNOSTIC &amp; INTERVENTION</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="14" customHeight="1">
-      <c r="A27" s="39" t="inlineStr">
+    <row r="36" ht="14" customHeight="1">
+      <c r="A36" s="39" t="inlineStr">
         <is>
           <t>SOPs applicables selon type incident — cocher les SOPs exécutées</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="48" t="inlineStr">
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="53" t="inlineStr">
         <is>
           <t>SOPs applicables (cocher) :   SOP-02 □   SOP-03 □   SOP-04 □   SOP-05 □   SOP-06 □   SOP-07 □   SOP-12 □</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="43" t="inlineStr">
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="48" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  SOP-02 — Vérification rack OOB</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="44" t="inlineStr">
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 1</t>
         </is>
       </c>
-      <c r="B30" s="45" t="inlineStr">
+      <c r="B39" s="50" t="inlineStr">
         <is>
           <t>Vérifier alimentation rack OOB sur chaque site (TH2, TH3, LF)</t>
         </is>
       </c>
-      <c r="C30" s="40" t="inlineStr">
+      <c r="C39" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D30" s="46" t="n"/>
-      <c r="E30" s="42" t="inlineStr">
+      <c r="D39" s="51" t="n"/>
+      <c r="E39" s="42" t="inlineStr">
         <is>
           <t>Outil : Visuel rack</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="44" t="inlineStr">
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 2</t>
         </is>
       </c>
-      <c r="B31" s="45" t="inlineStr">
+      <c r="B40" s="50" t="inlineStr">
         <is>
           <t>Vérifier chaque équipement OOB alimenté : switch, firewall</t>
         </is>
       </c>
-      <c r="C31" s="40" t="inlineStr">
+      <c r="C40" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D31" s="46" t="n"/>
-      <c r="E31" s="42" t="inlineStr">
+      <c r="D40" s="51" t="n"/>
+      <c r="E40" s="42" t="inlineStr">
         <is>
           <t>Outil : Visuel rack</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="44" t="inlineStr">
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 3</t>
         </is>
       </c>
-      <c r="B32" s="45" t="inlineStr">
+      <c r="B41" s="50" t="inlineStr">
         <is>
           <t>Consulter Vizee → onglet Firewall → état des liens opérateurs</t>
         </is>
       </c>
-      <c r="C32" s="40" t="inlineStr">
+      <c r="C41" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D32" s="46" t="n"/>
-      <c r="E32" s="42" t="inlineStr">
+      <c r="D41" s="51" t="n"/>
+      <c r="E41" s="42" t="inlineStr">
         <is>
           <t>Outil : Vizee</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="44" t="inlineStr">
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 4</t>
         </is>
       </c>
-      <c r="B33" s="45" t="inlineStr">
+      <c r="B42" s="50" t="inlineStr">
         <is>
           <t>Vérifier cablage fibre entre les switchs OOB</t>
         </is>
       </c>
-      <c r="C33" s="40" t="inlineStr">
+      <c r="C42" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D33" s="46" t="n"/>
-      <c r="E33" s="42" t="inlineStr">
+      <c r="D42" s="51" t="n"/>
+      <c r="E42" s="42" t="inlineStr">
         <is>
           <t>Outil : Visuel</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="44" t="inlineStr">
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 5</t>
         </is>
       </c>
-      <c r="B34" s="45" t="inlineStr">
+      <c r="B43" s="50" t="inlineStr">
         <is>
           <t>Vérifier cablage fibre entre switchs et PC supervision</t>
         </is>
       </c>
-      <c r="C34" s="40" t="inlineStr">
+      <c r="C43" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D34" s="46" t="n"/>
-      <c r="E34" s="42" t="inlineStr">
+      <c r="D43" s="51" t="n"/>
+      <c r="E43" s="42" t="inlineStr">
         <is>
           <t>Outil : Visuel</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="44" t="inlineStr">
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 6</t>
         </is>
       </c>
-      <c r="B35" s="45" t="inlineStr">
+      <c r="B44" s="50" t="inlineStr">
         <is>
           <t>Tester fibre à la caméra si suspicion salissure</t>
         </is>
       </c>
-      <c r="C35" s="40" t="inlineStr">
+      <c r="C44" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D35" s="46" t="n"/>
-      <c r="E35" s="42" t="inlineStr">
+      <c r="D44" s="51" t="n"/>
+      <c r="E44" s="42" t="inlineStr">
         <is>
           <t>Outil : Caméra inspection</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="40" t="inlineStr">
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="40" t="inlineStr">
         <is>
           <t>Cause identifiée</t>
         </is>
       </c>
-      <c r="B36" s="46" t="n"/>
-      <c r="C36" s="40" t="inlineStr">
+      <c r="B45" s="51" t="n"/>
+      <c r="C45" s="40" t="inlineStr">
         <is>
           <t>Action corrective réalisée</t>
         </is>
       </c>
-      <c r="D36" s="46" t="n"/>
-      <c r="E36" s="37" t="n"/>
-    </row>
-    <row r="37" ht="4" customHeight="1">
-      <c r="A37" s="37" t="n"/>
-      <c r="B37" s="37" t="n"/>
-      <c r="C37" s="37" t="n"/>
-      <c r="D37" s="37" t="n"/>
-      <c r="E37" s="37" t="n"/>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="43" t="inlineStr">
+      <c r="D45" s="51" t="n"/>
+      <c r="E45" s="37" t="n"/>
+    </row>
+    <row r="46" ht="4" customHeight="1">
+      <c r="A46" s="37" t="n"/>
+      <c r="B46" s="37" t="n"/>
+      <c r="C46" s="37" t="n"/>
+      <c r="D46" s="37" t="n"/>
+      <c r="E46" s="37" t="n"/>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="48" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  SOP-03 — Vérification supervision Lightsoft</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="44" t="inlineStr">
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 1</t>
         </is>
       </c>
-      <c r="B39" s="45" t="inlineStr">
+      <c r="B48" s="50" t="inlineStr">
         <is>
           <t>Vérifier que la session Lightsoft est active (pas de compte bloqué)</t>
         </is>
       </c>
-      <c r="C39" s="40" t="inlineStr">
+      <c r="C48" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D39" s="46" t="n"/>
-      <c r="E39" s="42" t="inlineStr">
+      <c r="D48" s="51" t="n"/>
+      <c r="E48" s="42" t="inlineStr">
         <is>
           <t>Outil : Lightsoft</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="44" t="inlineStr">
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 2</t>
         </is>
       </c>
-      <c r="B40" s="45" t="inlineStr">
+      <c r="B49" s="50" t="inlineStr">
         <is>
           <t>Consulter Vizee → Radius Account → log des dernières sessions</t>
         </is>
       </c>
-      <c r="C40" s="40" t="inlineStr">
+      <c r="C49" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D40" s="46" t="n"/>
-      <c r="E40" s="42" t="inlineStr">
+      <c r="D49" s="51" t="n"/>
+      <c r="E49" s="42" t="inlineStr">
         <is>
           <t>Outil : Vizee</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="44" t="inlineStr">
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 3</t>
         </is>
       </c>
-      <c r="B41" s="45" t="inlineStr">
+      <c r="B50" s="50" t="inlineStr">
         <is>
           <t>Ouvrir Trail List → sélectionner parcours → icône 'S' → vérifier chemin trafic actif</t>
         </is>
       </c>
-      <c r="C41" s="40" t="inlineStr">
+      <c r="C50" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D41" s="46" t="n"/>
-      <c r="E41" s="42" t="inlineStr">
+      <c r="D50" s="51" t="n"/>
+      <c r="E50" s="42" t="inlineStr">
         <is>
           <t>Outil : Lightsoft</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="44" t="inlineStr">
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 4</t>
         </is>
       </c>
-      <c r="B42" s="45" t="inlineStr">
+      <c r="B51" s="50" t="inlineStr">
         <is>
           <t>Vérifier compteurs CRC sur interfaces des cartes LB/HB/VHB concernées</t>
         </is>
       </c>
-      <c r="C42" s="40" t="inlineStr">
+      <c r="C51" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D42" s="46" t="n"/>
-      <c r="E42" s="42" t="inlineStr">
+      <c r="D51" s="51" t="n"/>
+      <c r="E51" s="42" t="inlineStr">
         <is>
           <t>Outil : Lightsoft</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="44" t="inlineStr">
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 5</t>
         </is>
       </c>
-      <c r="B43" s="45" t="inlineStr">
+      <c r="B52" s="50" t="inlineStr">
         <is>
           <t>Confirmer auprès des autres sites que l'accès Lightsoft fonctionne</t>
         </is>
       </c>
-      <c r="C43" s="40" t="inlineStr">
+      <c r="C52" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D43" s="46" t="n"/>
-      <c r="E43" s="42" t="inlineStr">
+      <c r="D52" s="51" t="n"/>
+      <c r="E52" s="42" t="inlineStr">
         <is>
           <t>Outil : Lightsoft</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="40" t="inlineStr">
-        <is>
-          <t>Cause identifiée</t>
-        </is>
-      </c>
-      <c r="B44" s="46" t="n"/>
-      <c r="C44" s="40" t="inlineStr">
-        <is>
-          <t>Action corrective réalisée</t>
-        </is>
-      </c>
-      <c r="D44" s="46" t="n"/>
-      <c r="E44" s="37" t="n"/>
-    </row>
-    <row r="45" ht="4" customHeight="1">
-      <c r="A45" s="37" t="n"/>
-      <c r="B45" s="37" t="n"/>
-      <c r="C45" s="37" t="n"/>
-      <c r="D45" s="37" t="n"/>
-      <c r="E45" s="37" t="n"/>
-    </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▶  SOP-04 — Vérification bascule OLP + OSNR</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Étape 1</t>
-        </is>
-      </c>
-      <c r="B47" s="45" t="inlineStr">
-        <is>
-          <t>Ouvrir Trail List → sélectionner parcours → icône 'S' → vérifier chemin actif</t>
-        </is>
-      </c>
-      <c r="C47" s="40" t="inlineStr">
-        <is>
-          <t>Résultat / Observation :</t>
-        </is>
-      </c>
-      <c r="D47" s="46" t="n"/>
-      <c r="E47" s="42" t="inlineStr">
-        <is>
-          <t>Outil : Lightsoft</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Étape 2</t>
-        </is>
-      </c>
-      <c r="B48" s="45" t="inlineStr">
-        <is>
-          <t>Confirmer bascule OLP : lien HS = rouge, lien en service = vert</t>
-        </is>
-      </c>
-      <c r="C48" s="40" t="inlineStr">
-        <is>
-          <t>Résultat / Observation :</t>
-        </is>
-      </c>
-      <c r="D48" s="46" t="n"/>
-      <c r="E48" s="42" t="inlineStr">
-        <is>
-          <t>Outil : Lightsoft</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Étape 3</t>
-        </is>
-      </c>
-      <c r="B49" s="45" t="inlineStr">
-        <is>
-          <t>Vérifier OSNR sur les 2 ports de réception des liens opérateurs</t>
-        </is>
-      </c>
-      <c r="C49" s="40" t="inlineStr">
-        <is>
-          <t>Résultat / Observation :</t>
-        </is>
-      </c>
-      <c r="D49" s="46" t="n"/>
-      <c r="E49" s="42" t="inlineStr">
-        <is>
-          <t>Outil : Lightsoft</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Étape 4</t>
-        </is>
-      </c>
-      <c r="B50" s="45" t="inlineStr">
-        <is>
-          <t>Vérifier état port OSC port 0 carte OADVLF (SFP OSC)</t>
-        </is>
-      </c>
-      <c r="C50" s="40" t="inlineStr">
-        <is>
-          <t>Résultat / Observation :</t>
-        </is>
-      </c>
-      <c r="D50" s="46" t="n"/>
-      <c r="E50" s="42" t="inlineStr">
-        <is>
-          <t>Outil : Lightsoft</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Étape 5</t>
-        </is>
-      </c>
-      <c r="B51" s="45" t="inlineStr">
-        <is>
-          <t>Si bascule OLP active → confirmer stabilité du lien restant</t>
-        </is>
-      </c>
-      <c r="C51" s="40" t="inlineStr">
-        <is>
-          <t>Résultat / Observation :</t>
-        </is>
-      </c>
-      <c r="D51" s="46" t="n"/>
-      <c r="E51" s="42" t="inlineStr">
-        <is>
-          <t>Outil : Lightsoft</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Étape 6</t>
-        </is>
-      </c>
-      <c r="B52" s="45" t="inlineStr">
-        <is>
-          <t>Surveiller évolution OSNR dans les 15 minutes suivantes</t>
-        </is>
-      </c>
-      <c r="C52" s="40" t="inlineStr">
-        <is>
-          <t>Résultat / Observation :</t>
-        </is>
-      </c>
-      <c r="D52" s="46" t="n"/>
-      <c r="E52" s="42" t="inlineStr">
-        <is>
-          <t>Outil : Lightsoft / Vizee</t>
         </is>
       </c>
     </row>
@@ -7746,13 +7703,13 @@
           <t>Cause identifiée</t>
         </is>
       </c>
-      <c r="B53" s="46" t="n"/>
+      <c r="B53" s="51" t="n"/>
       <c r="C53" s="40" t="inlineStr">
         <is>
           <t>Action corrective réalisée</t>
         </is>
       </c>
-      <c r="D53" s="46" t="n"/>
+      <c r="D53" s="51" t="n"/>
       <c r="E53" s="37" t="n"/>
     </row>
     <row r="54" ht="4" customHeight="1">
@@ -7763,721 +7720,785 @@
       <c r="E54" s="37" t="n"/>
     </row>
     <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="43" t="inlineStr">
+      <c r="A55" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▶  SOP-04 — Vérification bascule OLP + OSNR</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Étape 1</t>
+        </is>
+      </c>
+      <c r="B56" s="50" t="inlineStr">
+        <is>
+          <t>Ouvrir Trail List → sélectionner parcours → icône 'S' → vérifier chemin actif</t>
+        </is>
+      </c>
+      <c r="C56" s="40" t="inlineStr">
+        <is>
+          <t>Résultat / Observation :</t>
+        </is>
+      </c>
+      <c r="D56" s="51" t="n"/>
+      <c r="E56" s="42" t="inlineStr">
+        <is>
+          <t>Outil : Lightsoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Étape 2</t>
+        </is>
+      </c>
+      <c r="B57" s="50" t="inlineStr">
+        <is>
+          <t>Confirmer bascule OLP : lien HS = rouge, lien en service = vert</t>
+        </is>
+      </c>
+      <c r="C57" s="40" t="inlineStr">
+        <is>
+          <t>Résultat / Observation :</t>
+        </is>
+      </c>
+      <c r="D57" s="51" t="n"/>
+      <c r="E57" s="42" t="inlineStr">
+        <is>
+          <t>Outil : Lightsoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Étape 3</t>
+        </is>
+      </c>
+      <c r="B58" s="50" t="inlineStr">
+        <is>
+          <t>Vérifier OSNR sur les 2 ports de réception des liens opérateurs</t>
+        </is>
+      </c>
+      <c r="C58" s="40" t="inlineStr">
+        <is>
+          <t>Résultat / Observation :</t>
+        </is>
+      </c>
+      <c r="D58" s="51" t="n"/>
+      <c r="E58" s="42" t="inlineStr">
+        <is>
+          <t>Outil : Lightsoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Étape 4</t>
+        </is>
+      </c>
+      <c r="B59" s="50" t="inlineStr">
+        <is>
+          <t>Vérifier état port OSC port 0 carte OADVLF (SFP OSC)</t>
+        </is>
+      </c>
+      <c r="C59" s="40" t="inlineStr">
+        <is>
+          <t>Résultat / Observation :</t>
+        </is>
+      </c>
+      <c r="D59" s="51" t="n"/>
+      <c r="E59" s="42" t="inlineStr">
+        <is>
+          <t>Outil : Lightsoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Étape 5</t>
+        </is>
+      </c>
+      <c r="B60" s="50" t="inlineStr">
+        <is>
+          <t>Si bascule OLP active → confirmer stabilité du lien restant</t>
+        </is>
+      </c>
+      <c r="C60" s="40" t="inlineStr">
+        <is>
+          <t>Résultat / Observation :</t>
+        </is>
+      </c>
+      <c r="D60" s="51" t="n"/>
+      <c r="E60" s="42" t="inlineStr">
+        <is>
+          <t>Outil : Lightsoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Étape 6</t>
+        </is>
+      </c>
+      <c r="B61" s="50" t="inlineStr">
+        <is>
+          <t>Surveiller évolution OSNR dans les 15 minutes suivantes</t>
+        </is>
+      </c>
+      <c r="C61" s="40" t="inlineStr">
+        <is>
+          <t>Résultat / Observation :</t>
+        </is>
+      </c>
+      <c r="D61" s="51" t="n"/>
+      <c r="E61" s="42" t="inlineStr">
+        <is>
+          <t>Outil : Lightsoft / Vizee</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="40" t="inlineStr">
+        <is>
+          <t>Cause identifiée</t>
+        </is>
+      </c>
+      <c r="B62" s="51" t="n"/>
+      <c r="C62" s="40" t="inlineStr">
+        <is>
+          <t>Action corrective réalisée</t>
+        </is>
+      </c>
+      <c r="D62" s="51" t="n"/>
+      <c r="E62" s="37" t="n"/>
+    </row>
+    <row r="63" ht="4" customHeight="1">
+      <c r="A63" s="37" t="n"/>
+      <c r="B63" s="37" t="n"/>
+      <c r="C63" s="37" t="n"/>
+      <c r="D63" s="37" t="n"/>
+      <c r="E63" s="37" t="n"/>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" s="48" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  SOP-05 — Vérification physique rack OTN</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="44" t="inlineStr">
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 1</t>
         </is>
       </c>
-      <c r="B56" s="45" t="inlineStr">
+      <c r="B65" s="50" t="inlineStr">
         <is>
           <t>Se rendre sur site ou demander intervention locale</t>
         </is>
       </c>
-      <c r="C56" s="40" t="inlineStr">
+      <c r="C65" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D56" s="46" t="n"/>
-      <c r="E56" s="42" t="inlineStr">
+      <c r="D65" s="51" t="n"/>
+      <c r="E65" s="42" t="inlineStr">
         <is>
           <t>Outil : Sur site</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="44" t="inlineStr">
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 2</t>
         </is>
       </c>
-      <c r="B57" s="45" t="inlineStr">
+      <c r="B66" s="50" t="inlineStr">
         <is>
           <t>Vérifier voyants de toutes les cartes du chassis impacté</t>
         </is>
       </c>
-      <c r="C57" s="40" t="inlineStr">
+      <c r="C66" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D57" s="46" t="n"/>
-      <c r="E57" s="42" t="inlineStr">
+      <c r="D66" s="51" t="n"/>
+      <c r="E66" s="42" t="inlineStr">
         <is>
           <t>Outil : Visuel rack</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="44" t="inlineStr">
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 3</t>
         </is>
       </c>
-      <c r="B58" s="45" t="inlineStr">
+      <c r="B67" s="50" t="inlineStr">
         <is>
           <t>Vérifier alimentation chassis : voyant power card allumé, rectifier actif</t>
         </is>
       </c>
-      <c r="C58" s="40" t="inlineStr">
+      <c r="C67" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D58" s="46" t="n"/>
-      <c r="E58" s="42" t="inlineStr">
+      <c r="D67" s="51" t="n"/>
+      <c r="E67" s="42" t="inlineStr">
         <is>
           <t>Outil : Visuel rack</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="A59" s="44" t="inlineStr">
+    <row r="68" ht="20" customHeight="1">
+      <c r="A68" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 4</t>
         </is>
       </c>
-      <c r="B59" s="45" t="inlineStr">
+      <c r="B68" s="50" t="inlineStr">
         <is>
           <t>Identifier la carte défectueuse par process d'élimination</t>
         </is>
       </c>
-      <c r="C59" s="40" t="inlineStr">
+      <c r="C68" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D59" s="46" t="n"/>
-      <c r="E59" s="42" t="inlineStr">
+      <c r="D68" s="51" t="n"/>
+      <c r="E68" s="42" t="inlineStr">
         <is>
           <t>Outil : Visuel rack</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="A60" s="44" t="inlineStr">
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 5</t>
         </is>
       </c>
-      <c r="B60" s="45" t="inlineStr">
+      <c r="B69" s="50" t="inlineStr">
         <is>
           <t>Photographier l'état avant toute intervention</t>
         </is>
       </c>
-      <c r="C60" s="40" t="inlineStr">
+      <c r="C69" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D60" s="46" t="n"/>
-      <c r="E60" s="42" t="inlineStr">
+      <c r="D69" s="51" t="n"/>
+      <c r="E69" s="42" t="inlineStr">
         <is>
           <t>Outil : Photo</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="40" t="inlineStr">
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="40" t="inlineStr">
         <is>
           <t>Cause identifiée</t>
         </is>
       </c>
-      <c r="B61" s="46" t="n"/>
-      <c r="C61" s="40" t="inlineStr">
+      <c r="B70" s="51" t="n"/>
+      <c r="C70" s="40" t="inlineStr">
         <is>
           <t>Action corrective réalisée</t>
         </is>
       </c>
-      <c r="D61" s="46" t="n"/>
-      <c r="E61" s="37" t="n"/>
-    </row>
-    <row r="62" ht="4" customHeight="1">
-      <c r="A62" s="37" t="n"/>
-      <c r="B62" s="37" t="n"/>
-      <c r="C62" s="37" t="n"/>
-      <c r="D62" s="37" t="n"/>
-      <c r="E62" s="37" t="n"/>
-    </row>
-    <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="43" t="inlineStr">
+      <c r="D70" s="51" t="n"/>
+      <c r="E70" s="37" t="n"/>
+    </row>
+    <row r="71" ht="4" customHeight="1">
+      <c r="A71" s="37" t="n"/>
+      <c r="B71" s="37" t="n"/>
+      <c r="C71" s="37" t="n"/>
+      <c r="D71" s="37" t="n"/>
+      <c r="E71" s="37" t="n"/>
+    </row>
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="48" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  SOP-06 — Vérification carte RCP</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="44" t="inlineStr">
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 1</t>
         </is>
       </c>
-      <c r="B64" s="45" t="inlineStr">
+      <c r="B73" s="50" t="inlineStr">
         <is>
           <t>Vérifier bascule automatique RCP A → RCP B (chassis 9608 = doublon, 9603 = pas de doublon)</t>
         </is>
       </c>
-      <c r="C64" s="40" t="inlineStr">
+      <c r="C73" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D64" s="46" t="n"/>
-      <c r="E64" s="42" t="inlineStr">
+      <c r="D73" s="51" t="n"/>
+      <c r="E73" s="42" t="inlineStr">
         <is>
           <t>Outil : Lightsoft</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="20" customHeight="1">
-      <c r="A65" s="44" t="inlineStr">
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 2</t>
         </is>
       </c>
-      <c r="B65" s="45" t="inlineStr">
+      <c r="B74" s="50" t="inlineStr">
         <is>
           <t>Si bascule non effectuée sur 9608 → demander bascule manuelle via Ribbon ou manager</t>
         </is>
       </c>
-      <c r="C65" s="40" t="inlineStr">
+      <c r="C74" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D65" s="46" t="n"/>
-      <c r="E65" s="42" t="inlineStr">
+      <c r="D74" s="51" t="n"/>
+      <c r="E74" s="42" t="inlineStr">
         <is>
           <t>Outil : Ribbon</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="20" customHeight="1">
-      <c r="A66" s="44" t="inlineStr">
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 3</t>
         </is>
       </c>
-      <c r="B66" s="45" t="inlineStr">
+      <c r="B75" s="50" t="inlineStr">
         <is>
           <t>Vérifier câblage cuivre entre carte RCP et switch OOB (patch panel)</t>
         </is>
       </c>
-      <c r="C66" s="40" t="inlineStr">
+      <c r="C75" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D66" s="46" t="n"/>
-      <c r="E66" s="42" t="inlineStr">
+      <c r="D75" s="51" t="n"/>
+      <c r="E75" s="42" t="inlineStr">
         <is>
           <t>Outil : Visuel</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="20" customHeight="1">
-      <c r="A67" s="44" t="inlineStr">
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 4</t>
         </is>
       </c>
-      <c r="B67" s="45" t="inlineStr">
+      <c r="B76" s="50" t="inlineStr">
         <is>
           <t>Vérifier câblage entre carte FAN et switch OOB si alarme simultanée FAN + RCP</t>
         </is>
       </c>
-      <c r="C67" s="40" t="inlineStr">
+      <c r="C76" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D67" s="46" t="n"/>
-      <c r="E67" s="42" t="inlineStr">
+      <c r="D76" s="51" t="n"/>
+      <c r="E76" s="42" t="inlineStr">
         <is>
           <t>Outil : Visuel</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="18" customHeight="1">
-      <c r="A68" s="40" t="inlineStr">
+    <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="40" t="inlineStr">
         <is>
           <t>Cause identifiée</t>
         </is>
       </c>
-      <c r="B68" s="46" t="n"/>
-      <c r="C68" s="40" t="inlineStr">
+      <c r="B77" s="51" t="n"/>
+      <c r="C77" s="40" t="inlineStr">
         <is>
           <t>Action corrective réalisée</t>
         </is>
       </c>
-      <c r="D68" s="46" t="n"/>
-      <c r="E68" s="37" t="n"/>
-    </row>
-    <row r="69" ht="4" customHeight="1">
-      <c r="A69" s="37" t="n"/>
-      <c r="B69" s="37" t="n"/>
-      <c r="C69" s="37" t="n"/>
-      <c r="D69" s="37" t="n"/>
-      <c r="E69" s="37" t="n"/>
-    </row>
-    <row r="70" ht="18" customHeight="1">
-      <c r="A70" s="43" t="inlineStr">
+      <c r="D77" s="51" t="n"/>
+      <c r="E77" s="37" t="n"/>
+    </row>
+    <row r="78" ht="4" customHeight="1">
+      <c r="A78" s="37" t="n"/>
+      <c r="B78" s="37" t="n"/>
+      <c r="C78" s="37" t="n"/>
+      <c r="D78" s="37" t="n"/>
+      <c r="E78" s="37" t="n"/>
+    </row>
+    <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="48" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  SOP-07 — Vérification port SFP + jarretière</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="20" customHeight="1">
-      <c r="A71" s="44" t="inlineStr">
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 1</t>
         </is>
       </c>
-      <c r="B71" s="45" t="inlineStr">
+      <c r="B80" s="50" t="inlineStr">
         <is>
           <t>Vérifier état du SFP sur Lightsoft : valeur signal, erreurs</t>
         </is>
       </c>
-      <c r="C71" s="40" t="inlineStr">
+      <c r="C80" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D71" s="46" t="n"/>
-      <c r="E71" s="42" t="inlineStr">
+      <c r="D80" s="51" t="n"/>
+      <c r="E80" s="42" t="inlineStr">
         <is>
           <t>Outil : Lightsoft</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="20" customHeight="1">
-      <c r="A72" s="44" t="inlineStr">
+    <row r="81" ht="20" customHeight="1">
+      <c r="A81" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 2</t>
         </is>
       </c>
-      <c r="B72" s="45" t="inlineStr">
+      <c r="B81" s="50" t="inlineStr">
         <is>
           <t>Vérifier jarretière : bien connectée, non abîmée visuellement</t>
         </is>
       </c>
-      <c r="C72" s="40" t="inlineStr">
+      <c r="C81" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D72" s="46" t="n"/>
-      <c r="E72" s="42" t="inlineStr">
+      <c r="D81" s="51" t="n"/>
+      <c r="E81" s="42" t="inlineStr">
         <is>
           <t>Outil : Visuel</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="20" customHeight="1">
-      <c r="A73" s="44" t="inlineStr">
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 3</t>
         </is>
       </c>
-      <c r="B73" s="45" t="inlineStr">
+      <c r="B82" s="50" t="inlineStr">
         <is>
           <t>Inspecter jarretière à la caméra d'inspection fibre</t>
         </is>
       </c>
-      <c r="C73" s="40" t="inlineStr">
+      <c r="C82" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D73" s="46" t="n"/>
-      <c r="E73" s="42" t="inlineStr">
+      <c r="D82" s="51" t="n"/>
+      <c r="E82" s="42" t="inlineStr">
         <is>
           <t>Outil : Caméra inspection</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="20" customHeight="1">
-      <c r="A74" s="44" t="inlineStr">
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 4</t>
         </is>
       </c>
-      <c r="B74" s="45" t="inlineStr">
+      <c r="B83" s="50" t="inlineStr">
         <is>
           <t>Si salissure → nettoyage ou remplacement jarretière</t>
         </is>
       </c>
-      <c r="C74" s="40" t="inlineStr">
+      <c r="C83" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D74" s="46" t="n"/>
-      <c r="E74" s="42" t="inlineStr">
+      <c r="D83" s="51" t="n"/>
+      <c r="E83" s="42" t="inlineStr">
         <is>
           <t>Outil : Nettoyage fibre</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="44" t="inlineStr">
+    <row r="84" ht="20" customHeight="1">
+      <c r="A84" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 5</t>
         </is>
       </c>
-      <c r="B75" s="45" t="inlineStr">
+      <c r="B84" s="50" t="inlineStr">
         <is>
           <t>Vérifier aussi côté équipement opérateur si accès disponible</t>
         </is>
       </c>
-      <c r="C75" s="40" t="inlineStr">
+      <c r="C84" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D75" s="46" t="n"/>
-      <c r="E75" s="42" t="inlineStr">
+      <c r="D84" s="51" t="n"/>
+      <c r="E84" s="42" t="inlineStr">
         <is>
           <t>Outil : Site</t>
         </is>
       </c>
-    </row>
-    <row r="76" ht="18" customHeight="1">
-      <c r="A76" s="40" t="inlineStr">
-        <is>
-          <t>Cause identifiée</t>
-        </is>
-      </c>
-      <c r="B76" s="46" t="n"/>
-      <c r="C76" s="40" t="inlineStr">
-        <is>
-          <t>Action corrective réalisée</t>
-        </is>
-      </c>
-      <c r="D76" s="46" t="n"/>
-      <c r="E76" s="37" t="n"/>
-    </row>
-    <row r="77" ht="4" customHeight="1">
-      <c r="A77" s="37" t="n"/>
-      <c r="B77" s="37" t="n"/>
-      <c r="C77" s="37" t="n"/>
-      <c r="D77" s="37" t="n"/>
-      <c r="E77" s="37" t="n"/>
-    </row>
-    <row r="78" ht="18" customHeight="1">
-      <c r="A78" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▶  SOP-12 — Lecture PM Counters Lightsoft</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="20" customHeight="1">
-      <c r="A79" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Étape 1</t>
-        </is>
-      </c>
-      <c r="B79" s="45" t="inlineStr">
-        <is>
-          <t>Clic droit chassis → 'Open Shelf' → clic droit port → 'PMs' → 'Show port PMs'</t>
-        </is>
-      </c>
-      <c r="C79" s="40" t="inlineStr">
-        <is>
-          <t>Résultat / Observation :</t>
-        </is>
-      </c>
-      <c r="D79" s="46" t="n"/>
-      <c r="E79" s="42" t="inlineStr">
-        <is>
-          <t>Outil : Lightsoft</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="20" customHeight="1">
-      <c r="A80" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Étape 2</t>
-        </is>
-      </c>
-      <c r="B80" s="45" t="inlineStr">
-        <is>
-          <t>Vérifier OPR (puissance reçue) et OPT (puissance émise) en dBm</t>
-        </is>
-      </c>
-      <c r="C80" s="40" t="inlineStr">
-        <is>
-          <t>Résultat / Observation :</t>
-        </is>
-      </c>
-      <c r="D80" s="46" t="n"/>
-      <c r="E80" s="42" t="inlineStr">
-        <is>
-          <t>Outil : Lightsoft</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="20" customHeight="1">
-      <c r="A81" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Étape 3</t>
-        </is>
-      </c>
-      <c r="B81" s="45" t="inlineStr">
-        <is>
-          <t>Vérifier FEC Corrected / FEC Uncorrected — nombre élevé = dégradation critique</t>
-        </is>
-      </c>
-      <c r="C81" s="40" t="inlineStr">
-        <is>
-          <t>Résultat / Observation :</t>
-        </is>
-      </c>
-      <c r="D81" s="46" t="n"/>
-      <c r="E81" s="42" t="inlineStr">
-        <is>
-          <t>Outil : Lightsoft</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="20" customHeight="1">
-      <c r="A82" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Étape 4</t>
-        </is>
-      </c>
-      <c r="B82" s="45" t="inlineStr">
-        <is>
-          <t>Vérifier Pre-FEC BER et PCS Block Errors</t>
-        </is>
-      </c>
-      <c r="C82" s="40" t="inlineStr">
-        <is>
-          <t>Résultat / Observation :</t>
-        </is>
-      </c>
-      <c r="D82" s="46" t="n"/>
-      <c r="E82" s="42" t="inlineStr">
-        <is>
-          <t>Outil : Lightsoft</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="18" customHeight="1">
-      <c r="A83" s="40" t="inlineStr">
-        <is>
-          <t>Cause identifiée</t>
-        </is>
-      </c>
-      <c r="B83" s="46" t="n"/>
-      <c r="C83" s="40" t="inlineStr">
-        <is>
-          <t>Action corrective réalisée</t>
-        </is>
-      </c>
-      <c r="D83" s="46" t="n"/>
-      <c r="E83" s="37" t="n"/>
-    </row>
-    <row r="84" ht="4" customHeight="1">
-      <c r="A84" s="37" t="n"/>
-      <c r="B84" s="37" t="n"/>
-      <c r="C84" s="37" t="n"/>
-      <c r="D84" s="37" t="n"/>
-      <c r="E84" s="37" t="n"/>
     </row>
     <row r="85" ht="18" customHeight="1">
       <c r="A85" s="40" t="inlineStr">
         <is>
-          <t>Cause racine confirmée</t>
-        </is>
-      </c>
-      <c r="B85" s="41" t="n"/>
+          <t>Cause identifiée</t>
+        </is>
+      </c>
+      <c r="B85" s="51" t="n"/>
       <c r="C85" s="40" t="inlineStr">
         <is>
-          <t>Composant défectueux</t>
-        </is>
-      </c>
-      <c r="D85" s="41" t="n"/>
+          <t>Action corrective réalisée</t>
+        </is>
+      </c>
+      <c r="D85" s="51" t="n"/>
       <c r="E85" s="37" t="n"/>
     </row>
-    <row r="86" ht="6" customHeight="1">
+    <row r="86" ht="4" customHeight="1">
       <c r="A86" s="37" t="n"/>
       <c r="B86" s="37" t="n"/>
       <c r="C86" s="37" t="n"/>
       <c r="D86" s="37" t="n"/>
       <c r="E86" s="37" t="n"/>
     </row>
-    <row r="87" ht="22" customHeight="1">
-      <c r="A87" s="38" t="inlineStr">
-        <is>
-          <t>PHASE 3 — ESCALADE / RMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="14" customHeight="1">
-      <c r="A88" s="39" t="inlineStr">
-        <is>
-          <t>SOPs 08/09/10 · Ouverture tickets opérateur / Lugos / Ribbon</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="18" customHeight="1">
-      <c r="A89" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▶  SOP-08 — Ouverture ticket opérateur (Cogent / EuNetwork)</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="18" customHeight="1">
-      <c r="A90" s="40" t="inlineStr">
-        <is>
-          <t>Opérateur HS (via Vizee)</t>
-        </is>
-      </c>
-      <c r="B90" s="41" t="n"/>
+    <row r="87" ht="18" customHeight="1">
+      <c r="A87" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▶  SOP-12 — Lecture PM Counters Lightsoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="20" customHeight="1">
+      <c r="A88" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Étape 1</t>
+        </is>
+      </c>
+      <c r="B88" s="50" t="inlineStr">
+        <is>
+          <t>Clic droit chassis → 'Open Shelf' → clic droit port → 'PMs' → 'Show port PMs'</t>
+        </is>
+      </c>
+      <c r="C88" s="40" t="inlineStr">
+        <is>
+          <t>Résultat / Observation :</t>
+        </is>
+      </c>
+      <c r="D88" s="51" t="n"/>
+      <c r="E88" s="42" t="inlineStr">
+        <is>
+          <t>Outil : Lightsoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Étape 2</t>
+        </is>
+      </c>
+      <c r="B89" s="50" t="inlineStr">
+        <is>
+          <t>Vérifier OPR (puissance reçue) et OPT (puissance émise) en dBm</t>
+        </is>
+      </c>
+      <c r="C89" s="40" t="inlineStr">
+        <is>
+          <t>Résultat / Observation :</t>
+        </is>
+      </c>
+      <c r="D89" s="51" t="n"/>
+      <c r="E89" s="42" t="inlineStr">
+        <is>
+          <t>Outil : Lightsoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Étape 3</t>
+        </is>
+      </c>
+      <c r="B90" s="50" t="inlineStr">
+        <is>
+          <t>Vérifier FEC Corrected / FEC Uncorrected — nombre élevé = dégradation critique</t>
+        </is>
+      </c>
       <c r="C90" s="40" t="inlineStr">
         <is>
-          <t>Heure ouverture ticket</t>
-        </is>
-      </c>
-      <c r="D90" s="41" t="n"/>
-      <c r="E90" s="37" t="n"/>
-    </row>
-    <row r="91" ht="18" customHeight="1">
-      <c r="A91" s="40" t="inlineStr">
-        <is>
-          <t>N° ticket opérateur</t>
-        </is>
-      </c>
-      <c r="B91" s="41" t="n"/>
+          <t>Résultat / Observation :</t>
+        </is>
+      </c>
+      <c r="D90" s="51" t="n"/>
+      <c r="E90" s="42" t="inlineStr">
+        <is>
+          <t>Outil : Lightsoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Étape 4</t>
+        </is>
+      </c>
+      <c r="B91" s="50" t="inlineStr">
+        <is>
+          <t>Vérifier Pre-FEC BER et PCS Block Errors</t>
+        </is>
+      </c>
       <c r="C91" s="40" t="inlineStr">
         <is>
-          <t>Portail utilisé</t>
-        </is>
-      </c>
-      <c r="D91" s="41" t="n"/>
-      <c r="E91" s="37" t="n"/>
+          <t>Résultat / Observation :</t>
+        </is>
+      </c>
+      <c r="D91" s="51" t="n"/>
+      <c r="E91" s="42" t="inlineStr">
+        <is>
+          <t>Outil : Lightsoft</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="18" customHeight="1">
       <c r="A92" s="40" t="inlineStr">
         <is>
-          <t>Symptôme déclaré</t>
-        </is>
-      </c>
-      <c r="B92" s="41" t="n"/>
+          <t>Cause identifiée</t>
+        </is>
+      </c>
+      <c r="B92" s="51" t="n"/>
       <c r="C92" s="40" t="inlineStr">
         <is>
-          <t>Sites impactés déclarés</t>
-        </is>
-      </c>
-      <c r="D92" s="41" t="n"/>
+          <t>Action corrective réalisée</t>
+        </is>
+      </c>
+      <c r="D92" s="51" t="n"/>
       <c r="E92" s="37" t="n"/>
     </row>
-    <row r="93" ht="18" customHeight="1">
-      <c r="A93" s="40" t="inlineStr">
-        <is>
-          <t>Heure résolution opérateur</t>
-        </is>
-      </c>
-      <c r="B93" s="46" t="n"/>
-      <c r="C93" s="40" t="inlineStr">
-        <is>
-          <t>Confirmation reçue (O/N)</t>
-        </is>
-      </c>
-      <c r="D93" s="46" t="n"/>
+    <row r="93" ht="4" customHeight="1">
+      <c r="A93" s="37" t="n"/>
+      <c r="B93" s="37" t="n"/>
+      <c r="C93" s="37" t="n"/>
+      <c r="D93" s="37" t="n"/>
       <c r="E93" s="37" t="n"/>
     </row>
-    <row r="94" ht="4" customHeight="1">
-      <c r="A94" s="37" t="n"/>
-      <c r="B94" s="37" t="n"/>
-      <c r="C94" s="37" t="n"/>
-      <c r="D94" s="37" t="n"/>
+    <row r="94" ht="18" customHeight="1">
+      <c r="A94" s="40" t="inlineStr">
+        <is>
+          <t>Cause racine confirmée</t>
+        </is>
+      </c>
+      <c r="B94" s="41" t="n"/>
+      <c r="C94" s="40" t="inlineStr">
+        <is>
+          <t>Composant défectueux</t>
+        </is>
+      </c>
+      <c r="D94" s="41" t="n"/>
       <c r="E94" s="37" t="n"/>
     </row>
-    <row r="95" ht="18" customHeight="1">
-      <c r="A95" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▶  SOP-09 — Ouverture ticket Lugos</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="18" customHeight="1">
-      <c r="A96" s="40" t="inlineStr">
-        <is>
-          <t>Équipement OOB défaillant</t>
-        </is>
-      </c>
-      <c r="B96" s="41" t="n"/>
-      <c r="C96" s="40" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="D96" s="41" t="n"/>
-      <c r="E96" s="37" t="n"/>
-    </row>
-    <row r="97" ht="18" customHeight="1">
-      <c r="A97" s="40" t="inlineStr">
-        <is>
-          <t>N° ticket Lugos</t>
-        </is>
-      </c>
-      <c r="B97" s="41" t="n"/>
-      <c r="C97" s="40" t="inlineStr">
-        <is>
-          <t>Heure ouverture</t>
-        </is>
-      </c>
-      <c r="D97" s="41" t="n"/>
-      <c r="E97" s="37" t="n"/>
+    <row r="95" ht="6" customHeight="1">
+      <c r="A95" s="37" t="n"/>
+      <c r="B95" s="37" t="n"/>
+      <c r="C95" s="37" t="n"/>
+      <c r="D95" s="37" t="n"/>
+      <c r="E95" s="37" t="n"/>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="38" t="inlineStr">
+        <is>
+          <t>PHASE 3 — ESCALADE / RMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="14" customHeight="1">
+      <c r="A97" s="39" t="inlineStr">
+        <is>
+          <t>SOPs 08/09/10 · Ouverture tickets opérateur / Lugos / Ribbon</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="18" customHeight="1">
-      <c r="A98" s="40" t="inlineStr">
-        <is>
-          <t>Accès distant fourni (O/N)</t>
-        </is>
-      </c>
-      <c r="B98" s="46" t="n"/>
-      <c r="C98" s="40" t="inlineStr">
-        <is>
-          <t>Heure résolution</t>
-        </is>
-      </c>
-      <c r="D98" s="46" t="n"/>
-      <c r="E98" s="37" t="n"/>
-    </row>
-    <row r="99" ht="4" customHeight="1">
-      <c r="A99" s="37" t="n"/>
-      <c r="B99" s="37" t="n"/>
-      <c r="C99" s="37" t="n"/>
-      <c r="D99" s="37" t="n"/>
+      <c r="A98" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▶  SOP-08 — Ouverture ticket opérateur (Cogent / EuNetwork)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="18" customHeight="1">
+      <c r="A99" s="40" t="inlineStr">
+        <is>
+          <t>Opérateur HS (via Vizee)</t>
+        </is>
+      </c>
+      <c r="B99" s="41" t="n"/>
+      <c r="C99" s="40" t="inlineStr">
+        <is>
+          <t>Heure ouverture ticket</t>
+        </is>
+      </c>
+      <c r="D99" s="41" t="n"/>
       <c r="E99" s="37" t="n"/>
     </row>
     <row r="100" ht="18" customHeight="1">
-      <c r="A100" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▶  SOP-10 — Ouverture ticket Ribbon + RMA</t>
-        </is>
-      </c>
+      <c r="A100" s="40" t="inlineStr">
+        <is>
+          <t>N° ticket opérateur</t>
+        </is>
+      </c>
+      <c r="B100" s="41" t="n"/>
+      <c r="C100" s="40" t="inlineStr">
+        <is>
+          <t>Portail utilisé</t>
+        </is>
+      </c>
+      <c r="D100" s="41" t="n"/>
+      <c r="E100" s="37" t="n"/>
     </row>
     <row r="101" ht="18" customHeight="1">
       <c r="A101" s="40" t="inlineStr">
         <is>
-          <t>Numéro de série carte (Vizee)</t>
+          <t>Symptôme déclaré</t>
         </is>
       </c>
       <c r="B101" s="41" t="n"/>
       <c r="C101" s="40" t="inlineStr">
         <is>
-          <t>Type de carte / Chassis</t>
+          <t>Sites impactés déclarés</t>
         </is>
       </c>
       <c r="D101" s="41" t="n"/>
@@ -8486,831 +8507,922 @@
     <row r="102" ht="18" customHeight="1">
       <c r="A102" s="40" t="inlineStr">
         <is>
-          <t>N° ticket Ribbon</t>
-        </is>
-      </c>
-      <c r="B102" s="41" t="n"/>
+          <t>Heure résolution opérateur</t>
+        </is>
+      </c>
+      <c r="B102" s="51" t="n"/>
       <c r="C102" s="40" t="inlineStr">
         <is>
-          <t>Heure ouverture ticket Ribbon</t>
-        </is>
-      </c>
-      <c r="D102" s="41" t="n"/>
+          <t>Confirmation reçue (O/N)</t>
+        </is>
+      </c>
+      <c r="D102" s="51" t="n"/>
       <c r="E102" s="37" t="n"/>
     </row>
-    <row r="103" ht="18" customHeight="1">
-      <c r="A103" s="40" t="inlineStr">
-        <is>
-          <t>N° RMA</t>
-        </is>
-      </c>
-      <c r="B103" s="41" t="n"/>
-      <c r="C103" s="40" t="inlineStr">
-        <is>
-          <t>Date envoi RMA</t>
-        </is>
-      </c>
-      <c r="D103" s="41" t="n"/>
+    <row r="103" ht="4" customHeight="1">
+      <c r="A103" s="37" t="n"/>
+      <c r="B103" s="37" t="n"/>
+      <c r="C103" s="37" t="n"/>
+      <c r="D103" s="37" t="n"/>
       <c r="E103" s="37" t="n"/>
     </row>
     <row r="104" ht="18" customHeight="1">
-      <c r="A104" s="40" t="inlineStr">
-        <is>
-          <t>Service Delivery Ribbon contacté (O/N)</t>
-        </is>
-      </c>
-      <c r="B104" s="41" t="n"/>
-      <c r="C104" s="40" t="inlineStr">
-        <is>
-          <t>Nom interlocuteur Ribbon</t>
-        </is>
-      </c>
-      <c r="D104" s="41" t="n"/>
-      <c r="E104" s="37" t="n"/>
-    </row>
-    <row r="105" ht="16" customHeight="1">
-      <c r="A105" s="47" t="inlineStr">
-        <is>
-          <t>⚠  Changement carte OLP : remettre fibres à l'identique — pas de salissure</t>
-        </is>
-      </c>
+      <c r="A104" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▶  SOP-09 — Ouverture ticket Lugos</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="18" customHeight="1">
+      <c r="A105" s="40" t="inlineStr">
+        <is>
+          <t>Équipement OOB défaillant</t>
+        </is>
+      </c>
+      <c r="B105" s="41" t="n"/>
+      <c r="C105" s="40" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="D105" s="41" t="n"/>
+      <c r="E105" s="37" t="n"/>
     </row>
     <row r="106" ht="18" customHeight="1">
       <c r="A106" s="40" t="inlineStr">
         <is>
+          <t>N° ticket Lugos</t>
+        </is>
+      </c>
+      <c r="B106" s="41" t="n"/>
+      <c r="C106" s="40" t="inlineStr">
+        <is>
+          <t>Heure ouverture</t>
+        </is>
+      </c>
+      <c r="D106" s="41" t="n"/>
+      <c r="E106" s="37" t="n"/>
+    </row>
+    <row r="107" ht="18" customHeight="1">
+      <c r="A107" s="40" t="inlineStr">
+        <is>
+          <t>Accès distant fourni (O/N)</t>
+        </is>
+      </c>
+      <c r="B107" s="51" t="n"/>
+      <c r="C107" s="40" t="inlineStr">
+        <is>
+          <t>Heure résolution</t>
+        </is>
+      </c>
+      <c r="D107" s="51" t="n"/>
+      <c r="E107" s="37" t="n"/>
+    </row>
+    <row r="108" ht="4" customHeight="1">
+      <c r="A108" s="37" t="n"/>
+      <c r="B108" s="37" t="n"/>
+      <c r="C108" s="37" t="n"/>
+      <c r="D108" s="37" t="n"/>
+      <c r="E108" s="37" t="n"/>
+    </row>
+    <row r="109" ht="18" customHeight="1">
+      <c r="A109" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▶  SOP-10 — Ouverture ticket Ribbon + RMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="18" customHeight="1">
+      <c r="A110" s="40" t="inlineStr">
+        <is>
+          <t>Numéro de série carte (Vizee)</t>
+        </is>
+      </c>
+      <c r="B110" s="41" t="n"/>
+      <c r="C110" s="40" t="inlineStr">
+        <is>
+          <t>Type de carte / Chassis</t>
+        </is>
+      </c>
+      <c r="D110" s="41" t="n"/>
+      <c r="E110" s="37" t="n"/>
+    </row>
+    <row r="111" ht="18" customHeight="1">
+      <c r="A111" s="40" t="inlineStr">
+        <is>
+          <t>N° ticket Ribbon</t>
+        </is>
+      </c>
+      <c r="B111" s="41" t="n"/>
+      <c r="C111" s="40" t="inlineStr">
+        <is>
+          <t>Heure ouverture ticket Ribbon</t>
+        </is>
+      </c>
+      <c r="D111" s="41" t="n"/>
+      <c r="E111" s="37" t="n"/>
+    </row>
+    <row r="112" ht="18" customHeight="1">
+      <c r="A112" s="40" t="inlineStr">
+        <is>
+          <t>N° RMA</t>
+        </is>
+      </c>
+      <c r="B112" s="41" t="n"/>
+      <c r="C112" s="40" t="inlineStr">
+        <is>
+          <t>Date envoi RMA</t>
+        </is>
+      </c>
+      <c r="D112" s="41" t="n"/>
+      <c r="E112" s="37" t="n"/>
+    </row>
+    <row r="113" ht="18" customHeight="1">
+      <c r="A113" s="40" t="inlineStr">
+        <is>
+          <t>Service Delivery Ribbon contacté (O/N)</t>
+        </is>
+      </c>
+      <c r="B113" s="41" t="n"/>
+      <c r="C113" s="40" t="inlineStr">
+        <is>
+          <t>Nom interlocuteur Ribbon</t>
+        </is>
+      </c>
+      <c r="D113" s="41" t="n"/>
+      <c r="E113" s="37" t="n"/>
+    </row>
+    <row r="114" ht="16" customHeight="1">
+      <c r="A114" s="52" t="inlineStr">
+        <is>
+          <t>⚠  Changement carte OLP : remettre fibres à l'identique — pas de salissure</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="18" customHeight="1">
+      <c r="A115" s="40" t="inlineStr">
+        <is>
           <t>Heure résolution Ribbon</t>
         </is>
       </c>
-      <c r="B106" s="46" t="n"/>
-      <c r="C106" s="40" t="inlineStr">
+      <c r="B115" s="51" t="n"/>
+      <c r="C115" s="40" t="inlineStr">
         <is>
           <t>Confirmation clôture ticket (O/N)</t>
         </is>
       </c>
-      <c r="D106" s="46" t="n"/>
-      <c r="E106" s="37" t="n"/>
-    </row>
-    <row r="107" ht="6" customHeight="1">
-      <c r="A107" s="37" t="n"/>
-      <c r="B107" s="37" t="n"/>
-      <c r="C107" s="37" t="n"/>
-      <c r="D107" s="37" t="n"/>
-      <c r="E107" s="37" t="n"/>
-    </row>
-    <row r="108" ht="22" customHeight="1">
-      <c r="A108" s="38" t="inlineStr">
+      <c r="D115" s="51" t="n"/>
+      <c r="E115" s="37" t="n"/>
+    </row>
+    <row r="116" ht="6" customHeight="1">
+      <c r="A116" s="37" t="n"/>
+      <c r="B116" s="37" t="n"/>
+      <c r="C116" s="37" t="n"/>
+      <c r="D116" s="37" t="n"/>
+      <c r="E116" s="37" t="n"/>
+    </row>
+    <row r="117" ht="22" customHeight="1">
+      <c r="A117" s="38" t="inlineStr">
         <is>
           <t>PHASE 4 — COMMUNICATION</t>
         </is>
       </c>
     </row>
-    <row r="109" ht="14" customHeight="1">
-      <c r="A109" s="39" t="inlineStr">
+    <row r="118" ht="14" customHeight="1">
+      <c r="A118" s="39" t="inlineStr">
         <is>
           <t>SOP-11 · Informer toutes les parties prenantes</t>
         </is>
       </c>
     </row>
-    <row r="110" ht="18" customHeight="1">
-      <c r="A110" s="43" t="inlineStr">
+    <row r="119" ht="18" customHeight="1">
+      <c r="A119" s="48" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  SOP-11 — Communication incident</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="20" customHeight="1">
-      <c r="A111" s="44" t="inlineStr">
+    <row r="120" ht="20" customHeight="1">
+      <c r="A120" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 1</t>
         </is>
       </c>
-      <c r="B111" s="45" t="inlineStr">
+      <c r="B120" s="50" t="inlineStr">
         <is>
           <t>Informer immédiatement les autres sites de la situation</t>
         </is>
       </c>
-      <c r="C111" s="40" t="inlineStr">
+      <c r="C120" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D111" s="46" t="n"/>
-      <c r="E111" s="42" t="inlineStr">
+      <c r="D120" s="51" t="n"/>
+      <c r="E120" s="42" t="inlineStr">
         <is>
           <t>Outil : Téléphone / Teams</t>
         </is>
       </c>
     </row>
-    <row r="112" ht="20" customHeight="1">
-      <c r="A112" s="44" t="inlineStr">
+    <row r="121" ht="20" customHeight="1">
+      <c r="A121" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 2</t>
         </is>
       </c>
-      <c r="B112" s="45" t="inlineStr">
+      <c r="B121" s="50" t="inlineStr">
         <is>
           <t>Escalader auprès du manager (chaîne : TH3 → TH2 → LF)</t>
         </is>
       </c>
-      <c r="C112" s="40" t="inlineStr">
+      <c r="C121" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D112" s="46" t="n"/>
-      <c r="E112" s="42" t="inlineStr">
+      <c r="D121" s="51" t="n"/>
+      <c r="E121" s="42" t="inlineStr">
         <is>
           <t>Outil : Téléphone</t>
         </is>
       </c>
     </row>
-    <row r="113" ht="20" customHeight="1">
-      <c r="A113" s="44" t="inlineStr">
+    <row r="122" ht="20" customHeight="1">
+      <c r="A122" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 3</t>
         </is>
       </c>
-      <c r="B113" s="45" t="inlineStr">
+      <c r="B122" s="50" t="inlineStr">
         <is>
           <t>Si lien opérateur HS : informer Ribbon (ils ne peuvent plus accéder — info seulement)</t>
         </is>
       </c>
-      <c r="C113" s="40" t="inlineStr">
+      <c r="C122" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D113" s="46" t="n"/>
-      <c r="E113" s="42" t="inlineStr">
+      <c r="D122" s="51" t="n"/>
+      <c r="E122" s="42" t="inlineStr">
         <is>
           <t>Outil : Mail / Téléphone</t>
         </is>
       </c>
     </row>
-    <row r="114" ht="20" customHeight="1">
-      <c r="A114" s="44" t="inlineStr">
+    <row r="123" ht="20" customHeight="1">
+      <c r="A123" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 4</t>
         </is>
       </c>
-      <c r="B114" s="45" t="inlineStr">
+      <c r="B123" s="50" t="inlineStr">
         <is>
           <t>Envoyer mail d'incident : résumé étapes + liste clients impactés → paris OTN NOC + OTN management</t>
         </is>
       </c>
-      <c r="C114" s="40" t="inlineStr">
+      <c r="C123" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D114" s="46" t="n"/>
-      <c r="E114" s="42" t="inlineStr">
+      <c r="D123" s="51" t="n"/>
+      <c r="E123" s="42" t="inlineStr">
         <is>
           <t>Outil : Mail</t>
         </is>
       </c>
     </row>
-    <row r="115" ht="20" customHeight="1">
-      <c r="A115" s="44" t="inlineStr">
+    <row r="124" ht="20" customHeight="1">
+      <c r="A124" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 5</t>
         </is>
       </c>
-      <c r="B115" s="45" t="inlineStr">
+      <c r="B124" s="50" t="inlineStr">
         <is>
           <t>Mise à jour toutes les 30 min jusqu'à résolution</t>
         </is>
       </c>
-      <c r="C115" s="40" t="inlineStr">
+      <c r="C124" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D115" s="46" t="n"/>
-      <c r="E115" s="42" t="inlineStr">
+      <c r="D124" s="51" t="n"/>
+      <c r="E124" s="42" t="inlineStr">
         <is>
           <t>Outil : Mail / Teams</t>
         </is>
       </c>
     </row>
-    <row r="116" ht="20" customHeight="1">
-      <c r="A116" s="44" t="inlineStr">
+    <row r="125" ht="20" customHeight="1">
+      <c r="A125" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 6</t>
         </is>
       </c>
-      <c r="B116" s="45" t="inlineStr">
+      <c r="B125" s="50" t="inlineStr">
         <is>
           <t>Mail de clôture avec confirmation résolution + durée totale</t>
         </is>
       </c>
-      <c r="C116" s="40" t="inlineStr">
+      <c r="C125" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D116" s="46" t="n"/>
-      <c r="E116" s="42" t="inlineStr">
+      <c r="D125" s="51" t="n"/>
+      <c r="E125" s="42" t="inlineStr">
         <is>
           <t>Outil : Mail</t>
         </is>
       </c>
     </row>
-    <row r="117" ht="18" customHeight="1">
-      <c r="A117" s="40" t="inlineStr">
+    <row r="126" ht="18" customHeight="1">
+      <c r="A126" s="40" t="inlineStr">
         <is>
           <t>Sites informés (TH2/TH3/LF)</t>
         </is>
       </c>
-      <c r="B117" s="41" t="n"/>
-      <c r="C117" s="40" t="inlineStr">
+      <c r="B126" s="41" t="n"/>
+      <c r="C126" s="40" t="inlineStr">
         <is>
           <t>Heure information initiale</t>
         </is>
       </c>
-      <c r="D117" s="41" t="n"/>
-      <c r="E117" s="37" t="n"/>
-    </row>
-    <row r="118" ht="18" customHeight="1">
-      <c r="A118" s="40" t="inlineStr">
+      <c r="D126" s="41" t="n"/>
+      <c r="E126" s="37" t="n"/>
+    </row>
+    <row r="127" ht="18" customHeight="1">
+      <c r="A127" s="40" t="inlineStr">
         <is>
           <t>Manager informé</t>
         </is>
       </c>
-      <c r="B118" s="41" t="n"/>
-      <c r="C118" s="40" t="inlineStr">
+      <c r="B127" s="41" t="n"/>
+      <c r="C127" s="40" t="inlineStr">
         <is>
           <t>Canal utilisé</t>
         </is>
       </c>
-      <c r="D118" s="41" t="n"/>
-      <c r="E118" s="37" t="n"/>
-    </row>
-    <row r="119" ht="18" customHeight="1">
-      <c r="A119" s="40" t="inlineStr">
+      <c r="D127" s="41" t="n"/>
+      <c r="E127" s="37" t="n"/>
+    </row>
+    <row r="128" ht="18" customHeight="1">
+      <c r="A128" s="40" t="inlineStr">
         <is>
           <t>Ribbon informé (O/N)</t>
         </is>
       </c>
-      <c r="B119" s="41" t="n"/>
-      <c r="C119" s="40" t="inlineStr">
+      <c r="B128" s="41" t="n"/>
+      <c r="C128" s="40" t="inlineStr">
         <is>
           <t>Heure</t>
         </is>
       </c>
-      <c r="D119" s="41" t="n"/>
-      <c r="E119" s="37" t="n"/>
-    </row>
-    <row r="120" ht="18" customHeight="1">
-      <c r="A120" s="40" t="inlineStr">
+      <c r="D128" s="41" t="n"/>
+      <c r="E128" s="37" t="n"/>
+    </row>
+    <row r="129" ht="18" customHeight="1">
+      <c r="A129" s="40" t="inlineStr">
         <is>
           <t>Mail incident envoyé (O/N)</t>
         </is>
       </c>
-      <c r="B120" s="41" t="n"/>
-      <c r="C120" s="40" t="inlineStr">
+      <c r="B129" s="41" t="n"/>
+      <c r="C129" s="40" t="inlineStr">
         <is>
           <t>Heure envoi mail</t>
         </is>
       </c>
-      <c r="D120" s="41" t="n"/>
-      <c r="E120" s="37" t="n"/>
-    </row>
-    <row r="121" ht="18" customHeight="1">
-      <c r="A121" s="40" t="inlineStr">
-        <is>
-          <t>Nb mises à jour 30min envoyées</t>
-        </is>
-      </c>
-      <c r="B121" s="46" t="n"/>
-      <c r="C121" s="40" t="inlineStr">
+      <c r="D129" s="41" t="n"/>
+      <c r="E129" s="37" t="n"/>
+    </row>
+    <row r="130" ht="18" customHeight="1">
+      <c r="A130" s="40" t="inlineStr">
+        <is>
+          <t>Nb mises à jour 30min</t>
+        </is>
+      </c>
+      <c r="B130" s="51" t="n"/>
+      <c r="C130" s="40" t="inlineStr">
         <is>
           <t>Mail clôture envoyé (O/N)</t>
         </is>
       </c>
-      <c r="D121" s="46" t="n"/>
-      <c r="E121" s="37" t="n"/>
-    </row>
-    <row r="122" ht="6" customHeight="1">
-      <c r="A122" s="37" t="n"/>
-      <c r="B122" s="37" t="n"/>
-      <c r="C122" s="37" t="n"/>
-      <c r="D122" s="37" t="n"/>
-      <c r="E122" s="37" t="n"/>
-    </row>
-    <row r="123" ht="22" customHeight="1">
-      <c r="A123" s="38" t="inlineStr">
+      <c r="D130" s="51" t="n"/>
+      <c r="E130" s="37" t="n"/>
+    </row>
+    <row r="131" ht="6" customHeight="1">
+      <c r="A131" s="37" t="n"/>
+      <c r="B131" s="37" t="n"/>
+      <c r="C131" s="37" t="n"/>
+      <c r="D131" s="37" t="n"/>
+      <c r="E131" s="37" t="n"/>
+    </row>
+    <row r="132" ht="22" customHeight="1">
+      <c r="A132" s="38" t="inlineStr">
         <is>
           <t>PHASE 5 — VALIDATION POST-RÉSOLUTION</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="14" customHeight="1">
-      <c r="A124" s="39" t="inlineStr">
+    <row r="133" ht="14" customHeight="1">
+      <c r="A133" s="39" t="inlineStr">
         <is>
           <t>SOP-13 · Test Viavi OTU2 RFC 2544 · CRITIQUE uniquement</t>
         </is>
       </c>
     </row>
-    <row r="125" ht="18" customHeight="1">
-      <c r="A125" s="43" t="inlineStr">
+    <row r="134" ht="18" customHeight="1">
+      <c r="A134" s="48" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  SOP-13 — Validation post-résolution — Test Viavi OTU2 (RFC 2544)</t>
         </is>
       </c>
     </row>
-    <row r="126" ht="20" customHeight="1">
-      <c r="A126" s="44" t="inlineStr">
+    <row r="135" ht="20" customHeight="1">
+      <c r="A135" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 1</t>
         </is>
       </c>
-      <c r="B126" s="45" t="inlineStr">
+      <c r="B135" s="50" t="inlineStr">
         <is>
           <t>Connecter les 2 appareils Viavi à chaque extrémité du lien (TH2, TH3 ou LF)</t>
         </is>
       </c>
-      <c r="C126" s="40" t="inlineStr">
+      <c r="C135" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D126" s="46" t="n"/>
-      <c r="E126" s="42" t="inlineStr">
+      <c r="D135" s="51" t="n"/>
+      <c r="E135" s="42" t="inlineStr">
         <is>
           <t>Outil : Viavi / Sur site</t>
         </is>
       </c>
     </row>
-    <row r="127" ht="20" customHeight="1">
-      <c r="A127" s="44" t="inlineStr">
+    <row r="136" ht="20" customHeight="1">
+      <c r="A136" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 2</t>
         </is>
       </c>
-      <c r="B127" s="45" t="inlineStr">
+      <c r="B136" s="50" t="inlineStr">
         <is>
           <t>Configurer IP statique sur chaque Viavi (IP/Gateway/Masque/DNS)</t>
         </is>
       </c>
-      <c r="C127" s="40" t="inlineStr">
+      <c r="C136" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D127" s="46" t="n"/>
-      <c r="E127" s="42" t="inlineStr">
+      <c r="D136" s="51" t="n"/>
+      <c r="E136" s="42" t="inlineStr">
         <is>
           <t>Outil : Viavi</t>
         </is>
       </c>
     </row>
-    <row r="128" ht="20" customHeight="1">
-      <c r="A128" s="44" t="inlineStr">
+    <row r="137" ht="20" customHeight="1">
+      <c r="A137" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 3</t>
         </is>
       </c>
-      <c r="B128" s="45" t="inlineStr">
+      <c r="B137" s="50" t="inlineStr">
         <is>
           <t>Choisir le débit du test : 1G / 10G / 100G selon type lien OTU2</t>
         </is>
       </c>
-      <c r="C128" s="40" t="inlineStr">
+      <c r="C137" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D128" s="46" t="n"/>
-      <c r="E128" s="42" t="inlineStr">
+      <c r="D137" s="51" t="n"/>
+      <c r="E137" s="42" t="inlineStr">
         <is>
           <t>Outil : Viavi</t>
         </is>
       </c>
     </row>
-    <row r="129" ht="20" customHeight="1">
-      <c r="A129" s="44" t="inlineStr">
+    <row r="138" ht="20" customHeight="1">
+      <c r="A138" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 4</t>
         </is>
       </c>
-      <c r="B129" s="45" t="inlineStr">
+      <c r="B138" s="50" t="inlineStr">
         <is>
           <t>Activer le laser sur chaque Viavi — vérifier alignement optique (port local = vert)</t>
         </is>
       </c>
-      <c r="C129" s="40" t="inlineStr">
+      <c r="C138" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D129" s="46" t="n"/>
-      <c r="E129" s="42" t="inlineStr">
+      <c r="D138" s="51" t="n"/>
+      <c r="E138" s="42" t="inlineStr">
         <is>
           <t>Outil : Viavi</t>
         </is>
       </c>
     </row>
-    <row r="130" ht="20" customHeight="1">
-      <c r="A130" s="44" t="inlineStr">
+    <row r="139" ht="20" customHeight="1">
+      <c r="A139" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 5</t>
         </is>
       </c>
-      <c r="B130" s="45" t="inlineStr">
+      <c r="B139" s="50" t="inlineStr">
         <is>
           <t>Sélectionner RFC 2544 → Symétrique → mesures descendant et ascendant → Suivant</t>
         </is>
       </c>
-      <c r="C130" s="40" t="inlineStr">
+      <c r="C139" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D130" s="46" t="n"/>
-      <c r="E130" s="42" t="inlineStr">
+      <c r="D139" s="51" t="n"/>
+      <c r="E139" s="42" t="inlineStr">
         <is>
           <t>Outil : Viavi</t>
         </is>
       </c>
     </row>
-    <row r="131" ht="20" customHeight="1">
-      <c r="A131" s="44" t="inlineStr">
+    <row r="140" ht="20" customHeight="1">
+      <c r="A140" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 6</t>
         </is>
       </c>
-      <c r="B131" s="45" t="inlineStr">
+      <c r="B140" s="50" t="inlineStr">
         <is>
           <t>Sélectionner type de trame identique sur chaque Viavi → saisir les IP → Suivant</t>
         </is>
       </c>
-      <c r="C131" s="40" t="inlineStr">
+      <c r="C140" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D131" s="46" t="n"/>
-      <c r="E131" s="42" t="inlineStr">
+      <c r="D140" s="51" t="n"/>
+      <c r="E140" s="42" t="inlineStr">
         <is>
           <t>Outil : Viavi</t>
         </is>
       </c>
     </row>
-    <row r="132" ht="20" customHeight="1">
-      <c r="A132" s="44" t="inlineStr">
+    <row r="141" ht="20" customHeight="1">
+      <c r="A141" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 7</t>
         </is>
       </c>
-      <c r="B132" s="45" t="inlineStr">
+      <c r="B141" s="50" t="inlineStr">
         <is>
           <t>Saisir IP destination → Connexion au distant → attendre 'canal de communication = connecté'</t>
         </is>
       </c>
-      <c r="C132" s="40" t="inlineStr">
+      <c r="C141" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D132" s="46" t="n"/>
-      <c r="E132" s="42" t="inlineStr">
+      <c r="D141" s="51" t="n"/>
+      <c r="E141" s="42" t="inlineStr">
         <is>
           <t>Outil : Viavi</t>
         </is>
       </c>
     </row>
-    <row r="133" ht="20" customHeight="1">
-      <c r="A133" s="44" t="inlineStr">
+    <row r="142" ht="20" customHeight="1">
+      <c r="A142" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 8</t>
         </is>
       </c>
-      <c r="B133" s="45" t="inlineStr">
+      <c r="B142" s="50" t="inlineStr">
         <is>
           <t>Cliquer Suivant → attendre que 'Lancer le test' soit dégrisé → lancer le test</t>
         </is>
       </c>
-      <c r="C133" s="40" t="inlineStr">
+      <c r="C142" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D133" s="46" t="n"/>
-      <c r="E133" s="42" t="inlineStr">
+      <c r="D142" s="51" t="n"/>
+      <c r="E142" s="42" t="inlineStr">
         <is>
           <t>Outil : Viavi</t>
         </is>
       </c>
     </row>
-    <row r="134" ht="20" customHeight="1">
-      <c r="A134" s="44" t="inlineStr">
+    <row r="143" ht="20" customHeight="1">
+      <c r="A143" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 9</t>
         </is>
       </c>
-      <c r="B134" s="45" t="inlineStr">
+      <c r="B143" s="50" t="inlineStr">
         <is>
           <t>Vérifier résultats RFC 2544 : débit, latence, gigue, taux de perte — comparer SLA</t>
         </is>
       </c>
-      <c r="C134" s="40" t="inlineStr">
+      <c r="C143" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D134" s="46" t="n"/>
-      <c r="E134" s="42" t="inlineStr">
+      <c r="D143" s="51" t="n"/>
+      <c r="E143" s="42" t="inlineStr">
         <is>
           <t>Outil : Viavi / SLA</t>
         </is>
       </c>
     </row>
-    <row r="135" ht="20" customHeight="1">
-      <c r="A135" s="44" t="inlineStr">
+    <row r="144" ht="20" customHeight="1">
+      <c r="A144" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Étape 10</t>
         </is>
       </c>
-      <c r="B135" s="45" t="inlineStr">
+      <c r="B144" s="50" t="inlineStr">
         <is>
           <t>Confirmer résultats conformes avant de clôturer — joindre rapport Viavi au ticket Ribbon</t>
         </is>
       </c>
-      <c r="C135" s="40" t="inlineStr">
+      <c r="C144" s="40" t="inlineStr">
         <is>
           <t>Résultat / Observation :</t>
         </is>
       </c>
-      <c r="D135" s="46" t="n"/>
-      <c r="E135" s="42" t="inlineStr">
+      <c r="D144" s="51" t="n"/>
+      <c r="E144" s="42" t="inlineStr">
         <is>
           <t>Outil : Portail Ribbon / Mail</t>
         </is>
       </c>
-    </row>
-    <row r="136" ht="18" customHeight="1">
-      <c r="A136" s="40" t="inlineStr">
-        <is>
-          <t>Débit configuré (1G/10G/100G)</t>
-        </is>
-      </c>
-      <c r="B136" s="41" t="n"/>
-      <c r="C136" s="40" t="inlineStr">
-        <is>
-          <t>Extrémité 1 — Site / IP Viavi</t>
-        </is>
-      </c>
-      <c r="D136" s="41" t="n"/>
-      <c r="E136" s="37" t="n"/>
-    </row>
-    <row r="137" ht="18" customHeight="1">
-      <c r="A137" s="40" t="inlineStr">
-        <is>
-          <t>Extrémité 2 — Site / IP Viavi</t>
-        </is>
-      </c>
-      <c r="B137" s="41" t="n"/>
-      <c r="C137" s="40" t="inlineStr">
-        <is>
-          <t>Canal communication connecté (O/N)</t>
-        </is>
-      </c>
-      <c r="D137" s="41" t="n"/>
-      <c r="E137" s="37" t="n"/>
-    </row>
-    <row r="138" ht="16" customHeight="1">
-      <c r="A138" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Résultats RFC 2544</t>
-        </is>
-      </c>
-    </row>
-    <row r="139" ht="18" customHeight="1">
-      <c r="A139" s="40" t="inlineStr">
-        <is>
-          <t>Débit mesuré (Mbps)</t>
-        </is>
-      </c>
-      <c r="B139" s="46" t="n"/>
-      <c r="C139" s="40" t="inlineStr">
-        <is>
-          <t>Taux de perte paquet (%)</t>
-        </is>
-      </c>
-      <c r="D139" s="46" t="n"/>
-      <c r="E139" s="42" t="inlineStr">
-        <is>
-          <t>Seuil SLA : 0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="140" ht="18" customHeight="1">
-      <c r="A140" s="40" t="inlineStr">
-        <is>
-          <t>Latence aller-retour (ms)</t>
-        </is>
-      </c>
-      <c r="B140" s="46" t="n"/>
-      <c r="C140" s="40" t="inlineStr">
-        <is>
-          <t>Gigue (ms)</t>
-        </is>
-      </c>
-      <c r="D140" s="46" t="n"/>
-      <c r="E140" s="42" t="inlineStr">
-        <is>
-          <t>Seuil SLA selon contrat client</t>
-        </is>
-      </c>
-    </row>
-    <row r="141" ht="16" customHeight="1">
-      <c r="A141" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Mesures optiques (PM Counters Lightsoft)</t>
-        </is>
-      </c>
-    </row>
-    <row r="142" ht="18" customHeight="1">
-      <c r="A142" s="40" t="inlineStr">
-        <is>
-          <t>OSNR avant intervention (dB)</t>
-        </is>
-      </c>
-      <c r="B142" s="46" t="n"/>
-      <c r="C142" s="40" t="inlineStr">
-        <is>
-          <t>OSNR après intervention (dB)</t>
-        </is>
-      </c>
-      <c r="D142" s="46" t="n"/>
-      <c r="E142" s="37" t="n"/>
-    </row>
-    <row r="143" ht="18" customHeight="1">
-      <c r="A143" s="40" t="inlineStr">
-        <is>
-          <t>OPR avant (dBm)</t>
-        </is>
-      </c>
-      <c r="B143" s="46" t="n"/>
-      <c r="C143" s="40" t="inlineStr">
-        <is>
-          <t>OPR après (dBm)</t>
-        </is>
-      </c>
-      <c r="D143" s="46" t="n"/>
-      <c r="E143" s="37" t="n"/>
-    </row>
-    <row r="144" ht="18" customHeight="1">
-      <c r="A144" s="40" t="inlineStr">
-        <is>
-          <t>Pre-FEC BER</t>
-        </is>
-      </c>
-      <c r="B144" s="46" t="n"/>
-      <c r="C144" s="40" t="inlineStr">
-        <is>
-          <t>FEC Corrected / Uncorrected</t>
-        </is>
-      </c>
-      <c r="D144" s="46" t="n"/>
-      <c r="E144" s="37" t="n"/>
     </row>
     <row r="145" ht="18" customHeight="1">
       <c r="A145" s="40" t="inlineStr">
         <is>
-          <t>Résultat global (CONFORME/NON CONFORME)</t>
+          <t>Débit configuré (1G/10G/100G)</t>
         </is>
       </c>
       <c r="B145" s="41" t="n"/>
       <c r="C145" s="40" t="inlineStr">
         <is>
-          <t>Rapport Viavi joint (O/N)</t>
+          <t>Sites extrémités (Viavi 1 / Viavi 2)</t>
         </is>
       </c>
       <c r="D145" s="41" t="n"/>
       <c r="E145" s="37" t="n"/>
     </row>
     <row r="146" ht="16" customHeight="1">
-      <c r="A146" s="47" t="inlineStr">
-        <is>
-          <t>⚠  Si NON CONFORME : ne pas clôturer — rouvrir ticket Ribbon</t>
-        </is>
-      </c>
-    </row>
-    <row r="147" ht="6" customHeight="1">
-      <c r="A147" s="37" t="n"/>
-      <c r="B147" s="37" t="n"/>
-      <c r="C147" s="37" t="n"/>
-      <c r="D147" s="37" t="n"/>
-      <c r="E147" s="37" t="n"/>
-    </row>
-    <row r="148" ht="22" customHeight="1">
-      <c r="A148" s="38" t="inlineStr">
-        <is>
-          <t>CLÔTURE INCIDENT</t>
-        </is>
-      </c>
-    </row>
-    <row r="149" ht="18" customHeight="1">
-      <c r="A149" s="40" t="inlineStr">
-        <is>
-          <t>Heure clôture incident</t>
-        </is>
-      </c>
-      <c r="B149" s="41" t="n"/>
-      <c r="C149" s="40" t="inlineStr">
-        <is>
-          <t>Durée totale intervention (HH:MM)</t>
-        </is>
-      </c>
-      <c r="D149" s="41" t="n"/>
-      <c r="E149" s="37" t="n"/>
+      <c r="A146" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Résultats RFC 2544</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="18" customHeight="1">
+      <c r="A147" s="40" t="inlineStr">
+        <is>
+          <t>Débit mesuré (Mbps)</t>
+        </is>
+      </c>
+      <c r="B147" s="51" t="n"/>
+      <c r="C147" s="40" t="inlineStr">
+        <is>
+          <t>Taux de perte paquet (%)</t>
+        </is>
+      </c>
+      <c r="D147" s="51" t="n"/>
+      <c r="E147" s="42" t="inlineStr">
+        <is>
+          <t>Seuil SLA : 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="18" customHeight="1">
+      <c r="A148" s="40" t="inlineStr">
+        <is>
+          <t>Latence aller-retour (ms)</t>
+        </is>
+      </c>
+      <c r="B148" s="51" t="n"/>
+      <c r="C148" s="40" t="inlineStr">
+        <is>
+          <t>Gigue (ms)</t>
+        </is>
+      </c>
+      <c r="D148" s="51" t="n"/>
+      <c r="E148" s="42" t="inlineStr">
+        <is>
+          <t>Seuil SLA selon contrat</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="16" customHeight="1">
+      <c r="A149" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Mesures optiques (PM Counters Lightsoft)</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="18" customHeight="1">
       <c r="A150" s="40" t="inlineStr">
         <is>
-          <t>Statut final (RÉSOLU/PARTIEL/EN COURS)</t>
-        </is>
-      </c>
-      <c r="B150" s="41" t="n"/>
+          <t>OSNR avant (dB)</t>
+        </is>
+      </c>
+      <c r="B150" s="51" t="n"/>
       <c r="C150" s="40" t="inlineStr">
         <is>
-          <t>N° commit git (si modif workflow)</t>
-        </is>
-      </c>
-      <c r="D150" s="41" t="n"/>
+          <t>OSNR après (dB)</t>
+        </is>
+      </c>
+      <c r="D150" s="51" t="n"/>
       <c r="E150" s="37" t="n"/>
     </row>
     <row r="151" ht="18" customHeight="1">
       <c r="A151" s="40" t="inlineStr">
         <is>
+          <t>OPR avant (dBm)</t>
+        </is>
+      </c>
+      <c r="B151" s="51" t="n"/>
+      <c r="C151" s="40" t="inlineStr">
+        <is>
+          <t>OPR après (dBm)</t>
+        </is>
+      </c>
+      <c r="D151" s="51" t="n"/>
+      <c r="E151" s="37" t="n"/>
+    </row>
+    <row r="152" ht="18" customHeight="1">
+      <c r="A152" s="40" t="inlineStr">
+        <is>
+          <t>Pre-FEC BER</t>
+        </is>
+      </c>
+      <c r="B152" s="51" t="n"/>
+      <c r="C152" s="40" t="inlineStr">
+        <is>
+          <t>FEC Corrected / Uncorrected</t>
+        </is>
+      </c>
+      <c r="D152" s="51" t="n"/>
+      <c r="E152" s="37" t="n"/>
+    </row>
+    <row r="153" ht="18" customHeight="1">
+      <c r="A153" s="40" t="inlineStr">
+        <is>
+          <t>Résultat global (CONFORME / NON CONFORME)</t>
+        </is>
+      </c>
+      <c r="B153" s="41" t="n"/>
+      <c r="C153" s="40" t="inlineStr">
+        <is>
+          <t>Rapport Viavi joint (O/N)</t>
+        </is>
+      </c>
+      <c r="D153" s="41" t="n"/>
+      <c r="E153" s="37" t="n"/>
+    </row>
+    <row r="154" ht="16" customHeight="1">
+      <c r="A154" s="52" t="inlineStr">
+        <is>
+          <t>⚠  Si NON CONFORME : ne pas clôturer — rouvrir ticket Ribbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="6" customHeight="1">
+      <c r="A155" s="37" t="n"/>
+      <c r="B155" s="37" t="n"/>
+      <c r="C155" s="37" t="n"/>
+      <c r="D155" s="37" t="n"/>
+      <c r="E155" s="37" t="n"/>
+    </row>
+    <row r="156" ht="22" customHeight="1">
+      <c r="A156" s="38" t="inlineStr">
+        <is>
+          <t>CLÔTURE INCIDENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="18" customHeight="1">
+      <c r="A157" s="40" t="inlineStr">
+        <is>
+          <t>Heure clôture</t>
+        </is>
+      </c>
+      <c r="B157" s="41" t="n"/>
+      <c r="C157" s="40" t="inlineStr">
+        <is>
+          <t>Durée totale (HH:MM)</t>
+        </is>
+      </c>
+      <c r="D157" s="41" t="n"/>
+      <c r="E157" s="37" t="n"/>
+    </row>
+    <row r="158" ht="18" customHeight="1">
+      <c r="A158" s="40" t="inlineStr">
+        <is>
+          <t>Statut final (RÉSOLU / PARTIEL / EN COURS)</t>
+        </is>
+      </c>
+      <c r="B158" s="41" t="n"/>
+      <c r="C158" s="40" t="inlineStr">
+        <is>
+          <t>N° commit git si modif workflow</t>
+        </is>
+      </c>
+      <c r="D158" s="41" t="n"/>
+      <c r="E158" s="37" t="n"/>
+    </row>
+    <row r="159" ht="18" customHeight="1">
+      <c r="A159" s="40" t="inlineStr">
+        <is>
           <t>REX rédigé (O/N)</t>
         </is>
       </c>
-      <c r="B151" s="41" t="n"/>
-      <c r="C151" s="40" t="inlineStr">
-        <is>
-          <t>Chemin REX</t>
-        </is>
-      </c>
-      <c r="D151" s="41" t="n"/>
-      <c r="E151" s="42" t="inlineStr">
-        <is>
-          <t>docs/rex/REX-*.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="152" ht="40" customHeight="1">
-      <c r="A152" s="40" t="inlineStr">
+      <c r="B159" s="41" t="n"/>
+      <c r="C159" s="40" t="inlineStr">
+        <is>
+          <t>Chemin REX (docs/rex/REX-*.md)</t>
+        </is>
+      </c>
+      <c r="D159" s="41" t="n"/>
+      <c r="E159" s="37" t="n"/>
+    </row>
+    <row r="160" ht="48" customHeight="1">
+      <c r="A160" s="45" t="inlineStr">
         <is>
           <t>Observations / remarques libres</t>
         </is>
       </c>
-      <c r="B152" s="41" t="n"/>
-      <c r="C152" s="50" t="n"/>
-      <c r="E152" s="37" t="n"/>
+      <c r="B160" s="46" t="n"/>
+      <c r="E160" s="37" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="35">
-    <mergeCell ref="A148:E148"/>
+  <mergeCells count="43">
+    <mergeCell ref="A114:E114"/>
+    <mergeCell ref="A24:E24"/>
     <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A138:E138"/>
+    <mergeCell ref="A64:E64"/>
+    <mergeCell ref="A98:E98"/>
+    <mergeCell ref="B17:D17"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A123:E123"/>
-    <mergeCell ref="A88:E88"/>
-    <mergeCell ref="A70:E70"/>
-    <mergeCell ref="A110:E110"/>
+    <mergeCell ref="A132:E132"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A119:E119"/>
+    <mergeCell ref="A79:E79"/>
     <mergeCell ref="A146:E146"/>
-    <mergeCell ref="A124:E124"/>
     <mergeCell ref="A87:E87"/>
-    <mergeCell ref="A78:E78"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A16:E16"/>
-    <mergeCell ref="C152:D152"/>
-    <mergeCell ref="A108:E108"/>
-    <mergeCell ref="A46:E46"/>
-    <mergeCell ref="A89:E89"/>
-    <mergeCell ref="A27:E27"/>
-    <mergeCell ref="A105:E105"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A118:E118"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A133:E133"/>
+    <mergeCell ref="A149:E149"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="A154:E154"/>
     <mergeCell ref="A55:E55"/>
     <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A95:E95"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A104:E104"/>
+    <mergeCell ref="B160:D160"/>
+    <mergeCell ref="A47:E47"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A23:E23"/>
-    <mergeCell ref="A141:E141"/>
-    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A97:E97"/>
     <mergeCell ref="A109:E109"/>
-    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A35:E35"/>
     <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A100:E100"/>
+    <mergeCell ref="A156:E156"/>
     <mergeCell ref="A38:E38"/>
-    <mergeCell ref="A125:E125"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="A96:E96"/>
+    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="A134:E134"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="A117:E117"/>
+    <mergeCell ref="B21:D21"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"MINEUR,MAJEUR,CRITIQUE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>